<commit_message>
#4 R56 Resistor Edited in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/tracker-pro-airbnb-v1.0/BOM/eSpark_BOM_tracker-pro-airbnb-v1.0.xlsx
+++ b/Design-Files/tracker-pro-airbnb-v1.0/BOM/eSpark_BOM_tracker-pro-airbnb-v1.0.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2304" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2287" uniqueCount="659">
   <si>
     <t>Component list</t>
   </si>
@@ -1849,12 +1849,6 @@
     <t>F1, F2</t>
   </si>
   <si>
-    <t>P1, P2, P3, P4, P5, P6, P7, P8, P9, P10, P11, P12, P13, P14, P15, P16, P17, P18, P19</t>
-  </si>
-  <si>
-    <t>R4, R8, R11, R12, R13, R23, R24, R25, R27, R30, R31, R36, R41, R42, R44, R55, R68, R69</t>
-  </si>
-  <si>
     <t>R5, R6, R10, R39, R43, R57</t>
   </si>
   <si>
@@ -1927,9 +1921,6 @@
     <t>C57</t>
   </si>
   <si>
-    <t>R40, R56</t>
-  </si>
-  <si>
     <t>VMMC0571J150MV</t>
   </si>
   <si>
@@ -1984,12 +1975,6 @@
     <t>Custom Supplier Quote required</t>
   </si>
   <si>
-    <t>Flexible Ribbon Cable</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>SZYY0402YG</t>
   </si>
   <si>
@@ -2003,6 +1988,15 @@
   </si>
   <si>
     <t>C3, C5, C7, C8, C9, C11, C12, C13, C15, C16, C17, C24, C27, C28, C29, C34, C35, C37, C42, C45, C47, C59, C60, C73, C77, C79, C81, C82, C83</t>
+  </si>
+  <si>
+    <t>R4, R8, R11, R12, R13, R23, R24, R25, R27, R30, R31, R36, R41, R42, R44, R55, R56, R68, R69</t>
+  </si>
+  <si>
+    <t>R40</t>
+  </si>
+  <si>
+    <t>P1, P2, P3, P4, P5, P6, P7, P8, P9, P10, P11, P12, P13, P14, P15, P16, P17, P18, P19, P20</t>
   </si>
 </sst>
 </file>
@@ -3098,7 +3092,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AA129"/>
+  <dimension ref="A1:AA128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4" style="26" bestFit="1" customWidth="1"/>
@@ -3374,7 +3368,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>145</v>
@@ -3486,7 +3480,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="E12" s="50" t="s">
         <v>144</v>
@@ -3837,10 +3831,10 @@
         <v>390</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="J18" s="37" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="K18" s="37" t="s">
         <v>528</v>
@@ -4046,7 +4040,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="E22" s="37" t="s">
         <v>148</v>
@@ -4385,22 +4379,22 @@
         <v>54</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="F28" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G28" s="50" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="I28" s="50" t="s">
         <v>588</v>
       </c>
       <c r="J28" s="50" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="K28" s="50" t="s">
         <v>534</v>
@@ -5498,20 +5492,20 @@
         <v>72</v>
       </c>
       <c r="E48" s="50" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="F48" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G48" s="50" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="H48" s="50" t="s">
         <v>404</v>
       </c>
       <c r="I48" s="50"/>
       <c r="J48" s="50" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="K48" s="50" t="s">
         <v>588</v>
@@ -5724,10 +5718,10 @@
         <v>407</v>
       </c>
       <c r="I52" s="50" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="J52" s="50" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="K52" s="50"/>
       <c r="L52" s="50">
@@ -5904,7 +5898,7 @@
         <v>6</v>
       </c>
       <c r="O55" s="61" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="P55" s="38">
         <v>2.7</v>
@@ -6221,10 +6215,10 @@
         <v>413</v>
       </c>
       <c r="I61" s="37" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="J61" s="50" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="K61" s="50" t="s">
         <v>588</v>
@@ -6261,8 +6255,8 @@
       <c r="C62" s="53" t="s">
         <v>282</v>
       </c>
-      <c r="D62" s="68" t="s">
-        <v>609</v>
+      <c r="D62" s="66" t="s">
+        <v>658</v>
       </c>
       <c r="E62" s="66" t="s">
         <v>225</v>
@@ -6286,11 +6280,11 @@
         <v>588</v>
       </c>
       <c r="L62" s="66">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M62" s="66">
         <f>L62*5</f>
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="N62" s="66" t="s">
         <v>588</v>
@@ -6755,8 +6749,8 @@
       <c r="C71" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="D71" s="64" t="s">
-        <v>610</v>
+      <c r="D71" s="37" t="s">
+        <v>656</v>
       </c>
       <c r="E71" s="50" t="s">
         <v>199</v>
@@ -6778,11 +6772,11 @@
         <v>546</v>
       </c>
       <c r="L71" s="50">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M71" s="50">
         <f t="shared" ref="M71" si="58">L71*5</f>
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="N71" s="50">
         <v>100</v>
@@ -6810,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="D72" s="64" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="E72" s="50" t="s">
         <v>210</v>
@@ -7513,7 +7507,7 @@
         <v>27</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>635</v>
+        <v>657</v>
       </c>
       <c r="E85" s="50" t="s">
         <v>208</v>
@@ -7535,11 +7529,11 @@
         <v>546</v>
       </c>
       <c r="L85" s="50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M85" s="50">
         <f t="shared" ref="M85" si="71">L85*5</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N85" s="50">
         <v>100</v>
@@ -7636,10 +7630,10 @@
         <v>416</v>
       </c>
       <c r="I87" s="50" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="J87" s="50" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="K87" s="50" t="s">
         <v>557</v>
@@ -8271,7 +8265,7 @@
         <v>29</v>
       </c>
       <c r="D99" s="66" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E99" s="66" t="s">
         <v>224</v>
@@ -8329,22 +8323,22 @@
         <v>119</v>
       </c>
       <c r="E100" s="37" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="F100" s="37" t="s">
         <v>582</v>
       </c>
       <c r="G100" s="37" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="H100" s="37" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="I100" s="37" t="s">
         <v>588</v>
       </c>
       <c r="J100" s="37" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="K100" s="37" t="s">
         <v>588</v>
@@ -8385,20 +8379,20 @@
         <v>120</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F101" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G101" s="50" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="H101" s="50" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="I101" s="50"/>
       <c r="J101" s="50" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="K101" s="50" t="s">
         <v>588</v>
@@ -8732,7 +8726,7 @@
         <v>6</v>
       </c>
       <c r="O107" s="61" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="P107" s="51">
         <v>31.28</v>
@@ -8836,7 +8830,7 @@
         <v>6</v>
       </c>
       <c r="O109" s="61" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="P109" s="51">
         <v>6.7164999999999999</v>
@@ -8899,7 +8893,7 @@
         <v>6</v>
       </c>
       <c r="O110" s="61" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="P110" s="38">
         <v>10.1</v>
@@ -9246,13 +9240,13 @@
         <v>135</v>
       </c>
       <c r="E117" s="50" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="F117" s="50" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G117" s="50" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="H117" s="50" t="s">
         <v>421</v>
@@ -9261,7 +9255,7 @@
         <v>588</v>
       </c>
       <c r="J117" s="50" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="K117" s="50"/>
       <c r="L117" s="50">
@@ -9460,25 +9454,25 @@
         <v>139</v>
       </c>
       <c r="E121" s="50" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="F121" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G121" s="50" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="H121" s="50" t="s">
+        <v>629</v>
+      </c>
+      <c r="I121" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J121" s="50" t="s">
+        <v>628</v>
+      </c>
+      <c r="K121" s="50" t="s">
         <v>631</v>
-      </c>
-      <c r="I121" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J121" s="50" t="s">
-        <v>630</v>
-      </c>
-      <c r="K121" s="50" t="s">
-        <v>633</v>
       </c>
       <c r="L121" s="50">
         <v>1</v>
@@ -9618,19 +9612,19 @@
         <v>115</v>
       </c>
       <c r="C124" s="53" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D124" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E124" s="50" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="F124" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G124" s="50" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="H124" s="50" t="s">
         <v>588</v>
@@ -9655,7 +9649,7 @@
         <v>8</v>
       </c>
       <c r="O124" s="61" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="P124" s="51">
         <v>2.5</v>
@@ -9670,23 +9664,23 @@
     <row r="125" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1"/>
       <c r="B125" s="47">
-        <f t="shared" ref="B125:B127" si="112">ROW(B125) - ROW($B$9)</f>
+        <f t="shared" ref="B125:B126" si="112">ROW(B125) - ROW($B$9)</f>
         <v>116</v>
       </c>
       <c r="C125" s="53" t="s">
+        <v>615</v>
+      </c>
+      <c r="D125" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="E125" s="50" t="s">
+        <v>619</v>
+      </c>
+      <c r="F125" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="G125" s="50" t="s">
         <v>617</v>
-      </c>
-      <c r="D125" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E125" s="50" t="s">
-        <v>621</v>
-      </c>
-      <c r="F125" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G125" s="50" t="s">
-        <v>619</v>
       </c>
       <c r="H125" s="50" t="s">
         <v>588</v>
@@ -9714,7 +9708,7 @@
       <c r="P125" s="51"/>
       <c r="Q125" s="51"/>
       <c r="R125" s="65" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="S125" s="39"/>
     </row>
@@ -9725,19 +9719,19 @@
         <v>117</v>
       </c>
       <c r="C126" s="53" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E126" s="50" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="F126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G126" s="50" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H126" s="50" t="s">
         <v>588</v>
@@ -9765,118 +9759,69 @@
       <c r="P126" s="51"/>
       <c r="Q126" s="51"/>
       <c r="R126" s="65" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="S126" s="39"/>
     </row>
-    <row r="127" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1"/>
-      <c r="B127" s="47">
-        <f t="shared" si="112"/>
-        <v>118</v>
-      </c>
-      <c r="C127" s="53" t="s">
-        <v>617</v>
-      </c>
-      <c r="D127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E127" s="50"/>
-      <c r="F127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G127" s="50" t="s">
-        <v>654</v>
-      </c>
-      <c r="H127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="I127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="K127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="L127" s="50">
-        <v>1</v>
-      </c>
-      <c r="M127" s="50">
-        <f t="shared" ref="M127" si="113">L127*5</f>
+      <c r="B127" s="40"/>
+      <c r="C127" s="41"/>
+      <c r="D127" s="42"/>
+      <c r="E127" s="43"/>
+      <c r="F127" s="44"/>
+      <c r="G127" s="45"/>
+      <c r="H127" s="44"/>
+      <c r="I127" s="45"/>
+      <c r="J127" s="44"/>
+      <c r="K127" s="45"/>
+      <c r="L127" s="45"/>
+      <c r="M127" s="45"/>
+      <c r="N127" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="N127" s="50">
-        <v>6</v>
-      </c>
-      <c r="O127" s="61"/>
-      <c r="P127" s="51"/>
-      <c r="Q127" s="51"/>
-      <c r="R127" s="65" t="s">
-        <v>655</v>
-      </c>
-      <c r="S127" s="39"/>
+      <c r="O127" s="78"/>
+      <c r="P127" s="78"/>
+      <c r="Q127" s="48">
+        <f>SUM(Q11:Q126)</f>
+        <v>560.17779999999982</v>
+      </c>
+      <c r="R127" s="73"/>
+      <c r="S127" s="74"/>
     </row>
     <row r="128" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1"/>
-      <c r="B128" s="40"/>
-      <c r="C128" s="41"/>
-      <c r="D128" s="42"/>
-      <c r="E128" s="43"/>
-      <c r="F128" s="44"/>
-      <c r="G128" s="45"/>
-      <c r="H128" s="44"/>
-      <c r="I128" s="45"/>
-      <c r="J128" s="44"/>
-      <c r="K128" s="45"/>
-      <c r="L128" s="45"/>
-      <c r="M128" s="45"/>
+      <c r="B128" s="25"/>
+      <c r="C128" s="36"/>
+      <c r="D128" s="9"/>
+      <c r="E128" s="10"/>
+      <c r="F128" s="10"/>
+      <c r="G128" s="10"/>
+      <c r="H128" s="10"/>
+      <c r="I128" s="10"/>
+      <c r="J128" s="10"/>
+      <c r="K128" s="10"/>
+      <c r="L128" s="10"/>
+      <c r="M128" s="10"/>
       <c r="N128" s="77" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O128" s="78"/>
       <c r="P128" s="78"/>
-      <c r="Q128" s="48">
-        <f>SUM(Q11:Q127)</f>
-        <v>560.17779999999982</v>
-      </c>
-      <c r="R128" s="73"/>
-      <c r="S128" s="74"/>
-    </row>
-    <row r="129" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="1"/>
-      <c r="B129" s="25"/>
-      <c r="C129" s="36"/>
-      <c r="D129" s="9"/>
-      <c r="E129" s="10"/>
-      <c r="F129" s="10"/>
-      <c r="G129" s="10"/>
-      <c r="H129" s="10"/>
-      <c r="I129" s="10"/>
-      <c r="J129" s="10"/>
-      <c r="K129" s="10"/>
-      <c r="L129" s="10"/>
-      <c r="M129" s="10"/>
-      <c r="N129" s="77" t="s">
-        <v>6</v>
-      </c>
-      <c r="O129" s="78"/>
-      <c r="P129" s="78"/>
-      <c r="Q129" s="49">
-        <f>Q128/5</f>
+      <c r="Q128" s="49">
+        <f>Q127/5</f>
         <v>112.03555999999996</v>
       </c>
-      <c r="R129" s="75"/>
-      <c r="S129" s="76"/>
+      <c r="R128" s="75"/>
+      <c r="S128" s="76"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R128:S129"/>
+    <mergeCell ref="R127:S128"/>
+    <mergeCell ref="N127:P127"/>
     <mergeCell ref="N128:P128"/>
-    <mergeCell ref="N129:P129"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O11" r:id="rId1"/>
@@ -10000,7 +9945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S131"/>
+  <dimension ref="A1:S130"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -10275,7 +10220,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>145</v>
@@ -10387,7 +10332,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="E12" s="50" t="s">
         <v>144</v>
@@ -10738,10 +10683,10 @@
         <v>390</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="J18" s="37" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="K18" s="37" t="s">
         <v>528</v>
@@ -10947,7 +10892,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="E22" s="37" t="s">
         <v>148</v>
@@ -11286,22 +11231,22 @@
         <v>54</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="F28" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G28" s="50" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="I28" s="50" t="s">
         <v>588</v>
       </c>
       <c r="J28" s="50" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="K28" s="50" t="s">
         <v>534</v>
@@ -12399,20 +12344,20 @@
         <v>72</v>
       </c>
       <c r="E48" s="50" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="F48" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G48" s="50" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="H48" s="50" t="s">
         <v>404</v>
       </c>
       <c r="I48" s="50"/>
       <c r="J48" s="50" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="K48" s="50" t="s">
         <v>588</v>
@@ -12625,10 +12570,10 @@
         <v>407</v>
       </c>
       <c r="I52" s="50" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="J52" s="50" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="K52" s="50"/>
       <c r="L52" s="50">
@@ -12807,7 +12752,7 @@
         <v>11</v>
       </c>
       <c r="O55" s="61" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="P55" s="38">
         <v>2.7</v>
@@ -13124,10 +13069,10 @@
         <v>413</v>
       </c>
       <c r="I61" s="37" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="J61" s="50" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="K61" s="50" t="s">
         <v>588</v>
@@ -13164,8 +13109,8 @@
       <c r="C62" s="53" t="s">
         <v>282</v>
       </c>
-      <c r="D62" s="68" t="s">
-        <v>609</v>
+      <c r="D62" s="66" t="s">
+        <v>658</v>
       </c>
       <c r="E62" s="66" t="s">
         <v>225</v>
@@ -13189,14 +13134,14 @@
         <v>588</v>
       </c>
       <c r="L62" s="66">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M62" s="37">
         <f t="shared" si="1"/>
-        <v>190</v>
-      </c>
-      <c r="N62" s="50">
-        <v>15</v>
+        <v>200</v>
+      </c>
+      <c r="N62" s="50" t="s">
+        <v>588</v>
       </c>
       <c r="O62" s="66" t="s">
         <v>588</v>
@@ -13658,8 +13603,8 @@
       <c r="C71" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="D71" s="64" t="s">
-        <v>610</v>
+      <c r="D71" s="37" t="s">
+        <v>656</v>
       </c>
       <c r="E71" s="50" t="s">
         <v>199</v>
@@ -13681,11 +13626,11 @@
         <v>546</v>
       </c>
       <c r="L71" s="50">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M71" s="37">
         <f t="shared" si="1"/>
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="N71" s="37">
         <v>200</v>
@@ -13713,7 +13658,7 @@
         <v>27</v>
       </c>
       <c r="D72" s="64" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="E72" s="50" t="s">
         <v>210</v>
@@ -13738,7 +13683,7 @@
         <v>6</v>
       </c>
       <c r="M72" s="37">
-        <f t="shared" ref="M72:M127" si="30">L72*10</f>
+        <f t="shared" ref="M72:M126" si="30">L72*10</f>
         <v>60</v>
       </c>
       <c r="N72" s="50">
@@ -14416,7 +14361,7 @@
         <v>27</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>635</v>
+        <v>657</v>
       </c>
       <c r="E85" s="50" t="s">
         <v>208</v>
@@ -14438,11 +14383,11 @@
         <v>546</v>
       </c>
       <c r="L85" s="50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M85" s="37">
         <f t="shared" si="30"/>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N85" s="37">
         <v>100</v>
@@ -14539,10 +14484,10 @@
         <v>416</v>
       </c>
       <c r="I87" s="50" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="J87" s="50" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="K87" s="50" t="s">
         <v>557</v>
@@ -15174,7 +15119,7 @@
         <v>29</v>
       </c>
       <c r="D99" s="66" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E99" s="66" t="s">
         <v>224</v>
@@ -15232,22 +15177,22 @@
         <v>119</v>
       </c>
       <c r="E100" s="37" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="F100" s="37" t="s">
         <v>582</v>
       </c>
       <c r="G100" s="37" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="H100" s="37" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="I100" s="37" t="s">
         <v>588</v>
       </c>
       <c r="J100" s="37" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="K100" s="37" t="s">
         <v>588</v>
@@ -15288,20 +15233,20 @@
         <v>120</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F101" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G101" s="50" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="H101" s="50" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="I101" s="50"/>
       <c r="J101" s="50" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="K101" s="50" t="s">
         <v>588</v>
@@ -15621,7 +15566,7 @@
       </c>
       <c r="I107" s="50"/>
       <c r="J107" s="50" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="K107" s="50"/>
       <c r="L107" s="50">
@@ -15739,7 +15684,7 @@
         <v>11</v>
       </c>
       <c r="O109" s="61" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="P109" s="51">
         <v>6.7164999999999999</v>
@@ -15795,7 +15740,7 @@
         <v>11</v>
       </c>
       <c r="O110" s="61" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="P110" s="38">
         <v>10.1</v>
@@ -16142,13 +16087,13 @@
         <v>135</v>
       </c>
       <c r="E117" s="50" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="F117" s="50" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G117" s="50" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="H117" s="50" t="s">
         <v>421</v>
@@ -16157,7 +16102,7 @@
         <v>588</v>
       </c>
       <c r="J117" s="50" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="K117" s="50"/>
       <c r="L117" s="50">
@@ -16356,25 +16301,25 @@
         <v>139</v>
       </c>
       <c r="E121" s="50" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="F121" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G121" s="50" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="H121" s="50" t="s">
+        <v>629</v>
+      </c>
+      <c r="I121" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J121" s="50" t="s">
+        <v>628</v>
+      </c>
+      <c r="K121" s="50" t="s">
         <v>631</v>
-      </c>
-      <c r="I121" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J121" s="50" t="s">
-        <v>630</v>
-      </c>
-      <c r="K121" s="50" t="s">
-        <v>633</v>
       </c>
       <c r="L121" s="50">
         <v>1</v>
@@ -16514,19 +16459,19 @@
         <v>115</v>
       </c>
       <c r="C124" s="53" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D124" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E124" s="50" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="F124" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G124" s="50" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="H124" s="50" t="s">
         <v>588</v>
@@ -16551,7 +16496,7 @@
         <v>10</v>
       </c>
       <c r="O124" s="61" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="P124" s="51">
         <v>2.5</v>
@@ -16566,23 +16511,23 @@
     <row r="125" spans="1:19" s="60" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A125" s="59"/>
       <c r="B125" s="47">
-        <f t="shared" ref="B125:B127" si="52">ROW(B125) - ROW($B$9)</f>
+        <f t="shared" ref="B125:B126" si="52">ROW(B125) - ROW($B$9)</f>
         <v>116</v>
       </c>
       <c r="C125" s="53" t="s">
+        <v>615</v>
+      </c>
+      <c r="D125" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="E125" s="50" t="s">
+        <v>619</v>
+      </c>
+      <c r="F125" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="G125" s="50" t="s">
         <v>617</v>
-      </c>
-      <c r="D125" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E125" s="50" t="s">
-        <v>621</v>
-      </c>
-      <c r="F125" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G125" s="50" t="s">
-        <v>619</v>
       </c>
       <c r="H125" s="50" t="s">
         <v>588</v>
@@ -16610,30 +16555,30 @@
       <c r="P125" s="51"/>
       <c r="Q125" s="51"/>
       <c r="R125" s="65" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="S125" s="58"/>
     </row>
-    <row r="126" spans="1:19" s="60" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" s="60" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="59"/>
       <c r="B126" s="47">
         <f t="shared" si="52"/>
         <v>117</v>
       </c>
       <c r="C126" s="53" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E126" s="50" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="F126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G126" s="50" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H126" s="50" t="s">
         <v>588</v>
@@ -16661,121 +16606,72 @@
       <c r="P126" s="51"/>
       <c r="Q126" s="51"/>
       <c r="R126" s="65" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="S126" s="58"/>
     </row>
-    <row r="127" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1"/>
-      <c r="B127" s="47">
-        <f t="shared" si="52"/>
-        <v>118</v>
-      </c>
-      <c r="C127" s="53" t="s">
-        <v>617</v>
-      </c>
-      <c r="D127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E127" s="50"/>
-      <c r="F127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G127" s="50" t="s">
-        <v>654</v>
-      </c>
-      <c r="H127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="I127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="K127" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="L127" s="50">
-        <v>1</v>
-      </c>
-      <c r="M127" s="37">
-        <f t="shared" si="30"/>
-        <v>10</v>
-      </c>
-      <c r="N127" s="50">
-        <v>11</v>
-      </c>
-      <c r="O127" s="61"/>
-      <c r="P127" s="51"/>
-      <c r="Q127" s="51"/>
-      <c r="R127" s="65" t="s">
-        <v>655</v>
-      </c>
-      <c r="S127" s="39"/>
+      <c r="B127" s="40"/>
+      <c r="C127" s="41"/>
+      <c r="D127" s="42"/>
+      <c r="E127" s="43"/>
+      <c r="F127" s="44"/>
+      <c r="G127" s="45"/>
+      <c r="H127" s="44"/>
+      <c r="I127" s="45"/>
+      <c r="J127" s="44"/>
+      <c r="K127" s="45"/>
+      <c r="L127" s="45"/>
+      <c r="M127" s="45"/>
+      <c r="N127" s="77" t="s">
+        <v>5</v>
+      </c>
+      <c r="O127" s="78"/>
+      <c r="P127" s="78"/>
+      <c r="Q127" s="48">
+        <f>SUM(Q11:Q126)</f>
+        <v>628.29500000000007</v>
+      </c>
+      <c r="R127" s="45"/>
+      <c r="S127" s="45"/>
     </row>
     <row r="128" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1"/>
-      <c r="B128" s="40"/>
-      <c r="C128" s="41"/>
-      <c r="D128" s="42"/>
-      <c r="E128" s="43"/>
-      <c r="F128" s="44"/>
-      <c r="G128" s="45"/>
-      <c r="H128" s="44"/>
-      <c r="I128" s="45"/>
-      <c r="J128" s="44"/>
-      <c r="K128" s="45"/>
-      <c r="L128" s="45"/>
-      <c r="M128" s="45"/>
+      <c r="B128" s="25"/>
+      <c r="C128" s="36"/>
+      <c r="D128" s="9"/>
+      <c r="E128" s="10"/>
+      <c r="F128" s="10"/>
+      <c r="G128" s="10"/>
+      <c r="H128" s="10"/>
+      <c r="I128" s="10"/>
+      <c r="J128" s="10"/>
+      <c r="K128" s="10"/>
+      <c r="L128" s="10"/>
+      <c r="M128" s="10"/>
       <c r="N128" s="77" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O128" s="78"/>
       <c r="P128" s="78"/>
-      <c r="Q128" s="48">
-        <f>SUM(Q11:Q127)</f>
-        <v>628.29500000000007</v>
-      </c>
-      <c r="R128" s="45"/>
-      <c r="S128" s="45"/>
-    </row>
-    <row r="129" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q128" s="49">
+        <f>Q127/10</f>
+        <v>62.82950000000001</v>
+      </c>
+      <c r="R128" s="10"/>
+      <c r="S128" s="10"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
-      <c r="B129" s="25"/>
-      <c r="C129" s="36"/>
-      <c r="D129" s="9"/>
-      <c r="E129" s="10"/>
-      <c r="F129" s="10"/>
-      <c r="G129" s="10"/>
-      <c r="H129" s="10"/>
-      <c r="I129" s="10"/>
-      <c r="J129" s="10"/>
-      <c r="K129" s="10"/>
-      <c r="L129" s="10"/>
-      <c r="M129" s="10"/>
-      <c r="N129" s="77" t="s">
-        <v>6</v>
-      </c>
-      <c r="O129" s="78"/>
-      <c r="P129" s="78"/>
-      <c r="Q129" s="49">
-        <f>Q128/10</f>
-        <v>62.82950000000001</v>
-      </c>
-      <c r="R129" s="10"/>
-      <c r="S129" s="10"/>
-    </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="1"/>
-    </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A131" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="N127:P127"/>
     <mergeCell ref="N128:P128"/>
-    <mergeCell ref="N129:P129"/>
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
   </mergeCells>

</xml_diff>

<commit_message>
#4 SB5, SB6 Added in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/tracker-pro-airbnb-v1.0/BOM/eSpark_BOM_tracker-pro-airbnb-v1.0.xlsx
+++ b/Design-Files/tracker-pro-airbnb-v1.0/BOM/eSpark_BOM_tracker-pro-airbnb-v1.0.xlsx
@@ -1852,9 +1852,6 @@
     <t>R5, R6, R10, R39, R43, R57</t>
   </si>
   <si>
-    <t>SB1, SB2, SB3, SB4</t>
-  </si>
-  <si>
     <t>CC0201JRNPO8BN100</t>
   </si>
   <si>
@@ -1997,6 +1994,9 @@
   </si>
   <si>
     <t>P1, P2, P3, P4, P5, P6, P7, P8, P9, P10, P11, P12, P13, P14, P15, P16, P17, P18, P19, P20</t>
+  </si>
+  <si>
+    <t>SB1, SB2, SB3, SB4, SB5, SB6</t>
   </si>
 </sst>
 </file>
@@ -3368,7 +3368,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>145</v>
@@ -3480,7 +3480,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E12" s="50" t="s">
         <v>144</v>
@@ -3831,10 +3831,10 @@
         <v>390</v>
       </c>
       <c r="I18" s="37" t="s">
+        <v>610</v>
+      </c>
+      <c r="J18" s="37" t="s">
         <v>611</v>
-      </c>
-      <c r="J18" s="37" t="s">
-        <v>612</v>
       </c>
       <c r="K18" s="37" t="s">
         <v>528</v>
@@ -4040,7 +4040,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E22" s="37" t="s">
         <v>148</v>
@@ -4379,22 +4379,22 @@
         <v>54</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F28" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G28" s="50" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H28" s="50" t="s">
+        <v>639</v>
+      </c>
+      <c r="I28" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J28" s="50" t="s">
         <v>640</v>
-      </c>
-      <c r="I28" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J28" s="50" t="s">
-        <v>641</v>
       </c>
       <c r="K28" s="50" t="s">
         <v>534</v>
@@ -5492,20 +5492,20 @@
         <v>72</v>
       </c>
       <c r="E48" s="50" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F48" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G48" s="50" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H48" s="50" t="s">
         <v>404</v>
       </c>
       <c r="I48" s="50"/>
       <c r="J48" s="50" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="K48" s="50" t="s">
         <v>588</v>
@@ -5718,10 +5718,10 @@
         <v>407</v>
       </c>
       <c r="I52" s="50" t="s">
+        <v>612</v>
+      </c>
+      <c r="J52" s="50" t="s">
         <v>613</v>
-      </c>
-      <c r="J52" s="50" t="s">
-        <v>614</v>
       </c>
       <c r="K52" s="50"/>
       <c r="L52" s="50">
@@ -5898,7 +5898,7 @@
         <v>6</v>
       </c>
       <c r="O55" s="61" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P55" s="38">
         <v>2.7</v>
@@ -6215,10 +6215,10 @@
         <v>413</v>
       </c>
       <c r="I61" s="37" t="s">
+        <v>650</v>
+      </c>
+      <c r="J61" s="50" t="s">
         <v>651</v>
-      </c>
-      <c r="J61" s="50" t="s">
-        <v>652</v>
       </c>
       <c r="K61" s="50" t="s">
         <v>588</v>
@@ -6256,7 +6256,7 @@
         <v>282</v>
       </c>
       <c r="D62" s="66" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E62" s="66" t="s">
         <v>225</v>
@@ -6750,7 +6750,7 @@
         <v>27</v>
       </c>
       <c r="D71" s="37" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E71" s="50" t="s">
         <v>199</v>
@@ -7507,7 +7507,7 @@
         <v>27</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E85" s="50" t="s">
         <v>208</v>
@@ -7630,10 +7630,10 @@
         <v>416</v>
       </c>
       <c r="I87" s="50" t="s">
+        <v>620</v>
+      </c>
+      <c r="J87" s="50" t="s">
         <v>621</v>
-      </c>
-      <c r="J87" s="50" t="s">
-        <v>622</v>
       </c>
       <c r="K87" s="50" t="s">
         <v>557</v>
@@ -8265,7 +8265,7 @@
         <v>29</v>
       </c>
       <c r="D99" s="66" t="s">
-        <v>610</v>
+        <v>658</v>
       </c>
       <c r="E99" s="66" t="s">
         <v>224</v>
@@ -8289,11 +8289,11 @@
         <v>588</v>
       </c>
       <c r="L99" s="66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M99" s="66">
         <f t="shared" ref="M99" si="85">L99*5</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="N99" s="66" t="s">
         <v>588</v>
@@ -8323,22 +8323,22 @@
         <v>119</v>
       </c>
       <c r="E100" s="37" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F100" s="37" t="s">
         <v>582</v>
       </c>
       <c r="G100" s="37" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H100" s="37" t="s">
+        <v>642</v>
+      </c>
+      <c r="I100" s="37" t="s">
+        <v>588</v>
+      </c>
+      <c r="J100" s="37" t="s">
         <v>643</v>
-      </c>
-      <c r="I100" s="37" t="s">
-        <v>588</v>
-      </c>
-      <c r="J100" s="37" t="s">
-        <v>644</v>
       </c>
       <c r="K100" s="37" t="s">
         <v>588</v>
@@ -8379,20 +8379,20 @@
         <v>120</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F101" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G101" s="50" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H101" s="50" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I101" s="50"/>
       <c r="J101" s="50" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K101" s="50" t="s">
         <v>588</v>
@@ -8726,7 +8726,7 @@
         <v>6</v>
       </c>
       <c r="O107" s="61" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="P107" s="51">
         <v>31.28</v>
@@ -8830,7 +8830,7 @@
         <v>6</v>
       </c>
       <c r="O109" s="61" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="P109" s="51">
         <v>6.7164999999999999</v>
@@ -8893,7 +8893,7 @@
         <v>6</v>
       </c>
       <c r="O110" s="61" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="P110" s="38">
         <v>10.1</v>
@@ -9240,13 +9240,13 @@
         <v>135</v>
       </c>
       <c r="E117" s="50" t="s">
+        <v>623</v>
+      </c>
+      <c r="F117" s="50" t="s">
+        <v>647</v>
+      </c>
+      <c r="G117" s="50" t="s">
         <v>624</v>
-      </c>
-      <c r="F117" s="50" t="s">
-        <v>648</v>
-      </c>
-      <c r="G117" s="50" t="s">
-        <v>625</v>
       </c>
       <c r="H117" s="50" t="s">
         <v>421</v>
@@ -9255,7 +9255,7 @@
         <v>588</v>
       </c>
       <c r="J117" s="50" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="K117" s="50"/>
       <c r="L117" s="50">
@@ -9454,25 +9454,25 @@
         <v>139</v>
       </c>
       <c r="E121" s="50" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F121" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G121" s="50" t="s">
+        <v>629</v>
+      </c>
+      <c r="H121" s="50" t="s">
+        <v>628</v>
+      </c>
+      <c r="I121" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J121" s="50" t="s">
+        <v>627</v>
+      </c>
+      <c r="K121" s="50" t="s">
         <v>630</v>
-      </c>
-      <c r="H121" s="50" t="s">
-        <v>629</v>
-      </c>
-      <c r="I121" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J121" s="50" t="s">
-        <v>628</v>
-      </c>
-      <c r="K121" s="50" t="s">
-        <v>631</v>
       </c>
       <c r="L121" s="50">
         <v>1</v>
@@ -9612,19 +9612,19 @@
         <v>115</v>
       </c>
       <c r="C124" s="53" t="s">
+        <v>614</v>
+      </c>
+      <c r="D124" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="E124" s="50" t="s">
+        <v>648</v>
+      </c>
+      <c r="F124" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="G124" s="50" t="s">
         <v>615</v>
-      </c>
-      <c r="D124" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E124" s="50" t="s">
-        <v>649</v>
-      </c>
-      <c r="F124" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G124" s="50" t="s">
-        <v>616</v>
       </c>
       <c r="H124" s="50" t="s">
         <v>588</v>
@@ -9649,7 +9649,7 @@
         <v>8</v>
       </c>
       <c r="O124" s="61" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P124" s="51">
         <v>2.5</v>
@@ -9668,19 +9668,19 @@
         <v>116</v>
       </c>
       <c r="C125" s="53" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D125" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E125" s="50" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F125" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G125" s="50" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H125" s="50" t="s">
         <v>588</v>
@@ -9708,7 +9708,7 @@
       <c r="P125" s="51"/>
       <c r="Q125" s="51"/>
       <c r="R125" s="65" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S125" s="39"/>
     </row>
@@ -9719,19 +9719,19 @@
         <v>117</v>
       </c>
       <c r="C126" s="53" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E126" s="50" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G126" s="50" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H126" s="50" t="s">
         <v>588</v>
@@ -9759,7 +9759,7 @@
       <c r="P126" s="51"/>
       <c r="Q126" s="51"/>
       <c r="R126" s="65" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S126" s="39"/>
     </row>
@@ -10220,7 +10220,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>145</v>
@@ -10332,7 +10332,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E12" s="50" t="s">
         <v>144</v>
@@ -10683,10 +10683,10 @@
         <v>390</v>
       </c>
       <c r="I18" s="37" t="s">
+        <v>610</v>
+      </c>
+      <c r="J18" s="37" t="s">
         <v>611</v>
-      </c>
-      <c r="J18" s="37" t="s">
-        <v>612</v>
       </c>
       <c r="K18" s="37" t="s">
         <v>528</v>
@@ -10892,7 +10892,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E22" s="37" t="s">
         <v>148</v>
@@ -11231,22 +11231,22 @@
         <v>54</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F28" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G28" s="50" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H28" s="50" t="s">
+        <v>639</v>
+      </c>
+      <c r="I28" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J28" s="50" t="s">
         <v>640</v>
-      </c>
-      <c r="I28" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J28" s="50" t="s">
-        <v>641</v>
       </c>
       <c r="K28" s="50" t="s">
         <v>534</v>
@@ -12344,20 +12344,20 @@
         <v>72</v>
       </c>
       <c r="E48" s="50" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F48" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G48" s="50" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H48" s="50" t="s">
         <v>404</v>
       </c>
       <c r="I48" s="50"/>
       <c r="J48" s="50" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="K48" s="50" t="s">
         <v>588</v>
@@ -12570,10 +12570,10 @@
         <v>407</v>
       </c>
       <c r="I52" s="50" t="s">
+        <v>612</v>
+      </c>
+      <c r="J52" s="50" t="s">
         <v>613</v>
-      </c>
-      <c r="J52" s="50" t="s">
-        <v>614</v>
       </c>
       <c r="K52" s="50"/>
       <c r="L52" s="50">
@@ -12752,7 +12752,7 @@
         <v>11</v>
       </c>
       <c r="O55" s="61" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P55" s="38">
         <v>2.7</v>
@@ -13069,10 +13069,10 @@
         <v>413</v>
       </c>
       <c r="I61" s="37" t="s">
+        <v>650</v>
+      </c>
+      <c r="J61" s="50" t="s">
         <v>651</v>
-      </c>
-      <c r="J61" s="50" t="s">
-        <v>652</v>
       </c>
       <c r="K61" s="50" t="s">
         <v>588</v>
@@ -13110,7 +13110,7 @@
         <v>282</v>
       </c>
       <c r="D62" s="66" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E62" s="66" t="s">
         <v>225</v>
@@ -13604,7 +13604,7 @@
         <v>27</v>
       </c>
       <c r="D71" s="37" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E71" s="50" t="s">
         <v>199</v>
@@ -14361,7 +14361,7 @@
         <v>27</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E85" s="50" t="s">
         <v>208</v>
@@ -14484,10 +14484,10 @@
         <v>416</v>
       </c>
       <c r="I87" s="50" t="s">
+        <v>620</v>
+      </c>
+      <c r="J87" s="50" t="s">
         <v>621</v>
-      </c>
-      <c r="J87" s="50" t="s">
-        <v>622</v>
       </c>
       <c r="K87" s="50" t="s">
         <v>557</v>
@@ -15119,7 +15119,7 @@
         <v>29</v>
       </c>
       <c r="D99" s="66" t="s">
-        <v>610</v>
+        <v>658</v>
       </c>
       <c r="E99" s="66" t="s">
         <v>224</v>
@@ -15143,11 +15143,11 @@
         <v>588</v>
       </c>
       <c r="L99" s="66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M99" s="37">
         <f t="shared" si="30"/>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="N99" s="37">
         <v>50</v>
@@ -15177,22 +15177,22 @@
         <v>119</v>
       </c>
       <c r="E100" s="37" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F100" s="37" t="s">
         <v>582</v>
       </c>
       <c r="G100" s="37" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H100" s="37" t="s">
+        <v>642</v>
+      </c>
+      <c r="I100" s="37" t="s">
+        <v>588</v>
+      </c>
+      <c r="J100" s="37" t="s">
         <v>643</v>
-      </c>
-      <c r="I100" s="37" t="s">
-        <v>588</v>
-      </c>
-      <c r="J100" s="37" t="s">
-        <v>644</v>
       </c>
       <c r="K100" s="37" t="s">
         <v>588</v>
@@ -15233,20 +15233,20 @@
         <v>120</v>
       </c>
       <c r="E101" s="50" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F101" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G101" s="50" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H101" s="50" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I101" s="50"/>
       <c r="J101" s="50" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K101" s="50" t="s">
         <v>588</v>
@@ -15566,7 +15566,7 @@
       </c>
       <c r="I107" s="50"/>
       <c r="J107" s="50" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="K107" s="50"/>
       <c r="L107" s="50">
@@ -15684,7 +15684,7 @@
         <v>11</v>
       </c>
       <c r="O109" s="61" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="P109" s="51">
         <v>6.7164999999999999</v>
@@ -15740,7 +15740,7 @@
         <v>11</v>
       </c>
       <c r="O110" s="61" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="P110" s="38">
         <v>10.1</v>
@@ -16087,13 +16087,13 @@
         <v>135</v>
       </c>
       <c r="E117" s="50" t="s">
+        <v>623</v>
+      </c>
+      <c r="F117" s="50" t="s">
+        <v>647</v>
+      </c>
+      <c r="G117" s="50" t="s">
         <v>624</v>
-      </c>
-      <c r="F117" s="50" t="s">
-        <v>648</v>
-      </c>
-      <c r="G117" s="50" t="s">
-        <v>625</v>
       </c>
       <c r="H117" s="50" t="s">
         <v>421</v>
@@ -16102,7 +16102,7 @@
         <v>588</v>
       </c>
       <c r="J117" s="50" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="K117" s="50"/>
       <c r="L117" s="50">
@@ -16301,25 +16301,25 @@
         <v>139</v>
       </c>
       <c r="E121" s="50" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F121" s="50" t="s">
         <v>582</v>
       </c>
       <c r="G121" s="50" t="s">
+        <v>629</v>
+      </c>
+      <c r="H121" s="50" t="s">
+        <v>628</v>
+      </c>
+      <c r="I121" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="J121" s="50" t="s">
+        <v>627</v>
+      </c>
+      <c r="K121" s="50" t="s">
         <v>630</v>
-      </c>
-      <c r="H121" s="50" t="s">
-        <v>629</v>
-      </c>
-      <c r="I121" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="J121" s="50" t="s">
-        <v>628</v>
-      </c>
-      <c r="K121" s="50" t="s">
-        <v>631</v>
       </c>
       <c r="L121" s="50">
         <v>1</v>
@@ -16459,19 +16459,19 @@
         <v>115</v>
       </c>
       <c r="C124" s="53" t="s">
+        <v>614</v>
+      </c>
+      <c r="D124" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="E124" s="50" t="s">
+        <v>648</v>
+      </c>
+      <c r="F124" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="G124" s="50" t="s">
         <v>615</v>
-      </c>
-      <c r="D124" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="E124" s="50" t="s">
-        <v>649</v>
-      </c>
-      <c r="F124" s="50" t="s">
-        <v>588</v>
-      </c>
-      <c r="G124" s="50" t="s">
-        <v>616</v>
       </c>
       <c r="H124" s="50" t="s">
         <v>588</v>
@@ -16496,7 +16496,7 @@
         <v>10</v>
       </c>
       <c r="O124" s="61" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P124" s="51">
         <v>2.5</v>
@@ -16515,19 +16515,19 @@
         <v>116</v>
       </c>
       <c r="C125" s="53" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D125" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E125" s="50" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F125" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G125" s="50" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H125" s="50" t="s">
         <v>588</v>
@@ -16555,7 +16555,7 @@
       <c r="P125" s="51"/>
       <c r="Q125" s="51"/>
       <c r="R125" s="65" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S125" s="58"/>
     </row>
@@ -16566,19 +16566,19 @@
         <v>117</v>
       </c>
       <c r="C126" s="53" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="E126" s="50" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F126" s="50" t="s">
         <v>588</v>
       </c>
       <c r="G126" s="50" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H126" s="50" t="s">
         <v>588</v>
@@ -16606,7 +16606,7 @@
       <c r="P126" s="51"/>
       <c r="Q126" s="51"/>
       <c r="R126" s="65" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="S126" s="58"/>
     </row>

</xml_diff>